<commit_message>
docs: apresentacao em PDF, status final no README e correcao D1/Q1 na BOM.
</commit_message>
<xml_diff>
--- a/docs/datalogger.xlsx
+++ b/docs/datalogger.xlsx
@@ -299,7 +299,7 @@
     <t xml:space="preserve">Micro Commercial Components</t>
   </si>
   <si>
-    <t xml:space="preserve">Schottky de 40 V/1 A no caminho da bateria (seleção de fonte com o MOSFET Q1): queda baixa (~0,45 V) para aproveitar a LiPo. SOD-123 fácil de soldar.</t>
+    <t xml:space="preserve">Schottky que leva o VBUS (5 V do USB-C) ao barramento do sistema (VSYS); 40 V/1 A, queda ~0,45 V, folga para os 5 V. SOD-123 fácil de soldar.</t>
   </si>
   <si>
     <t xml:space="preserve">833-B5819W-TP</t>
@@ -659,7 +659,7 @@
     <t xml:space="preserve">Diodes Inc.</t>
   </si>
   <si>
-    <t xml:space="preserve">MOSFET P em função de diodo ideal na seleção USB × bateria (USB com prioridade): RDS(on) ~ 52 mΩ, queda muito menor que um diodo. SOT-23 fácil de soldar.</t>
+    <t xml:space="preserve">MOSFET P em função de diodo ideal para a bateria: conduz quando só há a LiPo e é bloqueado pelo VBUS quando a USB está ligada (prioridade da USB). RDS(on) ~ 52 mΩ: queda de poucos mV, aproveita toda a carga da bateria. SOT-23.</t>
   </si>
   <si>
     <t xml:space="preserve">621-DMG2305UX-13</t>
@@ -2611,7 +2611,7 @@
       </c>
       <c r="O20" s="5"/>
     </row>
-    <row r="21" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
         <v>205</v>
       </c>

</xml_diff>